<commit_message>
dr mujahid ganti semua index
</commit_message>
<xml_diff>
--- a/excel_outputs/pglib_opf_case57_ieee.xlsx
+++ b/excel_outputs/pglib_opf_case57_ieee.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\firda\belajar\ISE711\old\DCOPF-main\DCOPF-main\excel_outputs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\firda\belajar\ISE711\excel_outputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{212CC456-3249-498C-A4DC-F4F8C5DAC5AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2290007F-869F-4A59-94E1-EF60E8AC4A5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="53">
   <si>
     <t>bus_i</t>
   </si>
@@ -182,10 +182,7 @@
     <t>angmax</t>
   </si>
   <si>
-    <t>unique</t>
-  </si>
-  <si>
-    <t>zero or one</t>
+    <t>line_ID</t>
   </si>
 </sst>
 </file>
@@ -207,21 +204,15 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -244,30 +235,16 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3781,47 +3758,47 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
+      <c r="A1" t="s">
+        <v>52</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>51</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
@@ -3829,19 +3806,19 @@
         <v>1</v>
       </c>
       <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
         <v>2</v>
       </c>
-      <c r="C2">
+      <c r="D2">
         <v>8.3000000000000001E-3</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>2.8000000000000001E-2</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <v>0.129</v>
-      </c>
-      <c r="F2">
-        <v>1005</v>
       </c>
       <c r="G2">
         <v>1005</v>
@@ -3850,22 +3827,22 @@
         <v>1005</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>1005</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L2">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M2">
-        <v>30</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>53</v>
+        <v>-30</v>
+      </c>
+      <c r="N2">
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
@@ -3873,19 +3850,19 @@
         <v>2</v>
       </c>
       <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
         <v>3</v>
       </c>
-      <c r="C3">
+      <c r="D3">
         <v>2.98E-2</v>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>8.5000000000000006E-2</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <v>8.1799999999999998E-2</v>
-      </c>
-      <c r="F3">
-        <v>326</v>
       </c>
       <c r="G3">
         <v>326</v>
@@ -3894,18 +3871,21 @@
         <v>326</v>
       </c>
       <c r="I3">
-        <v>0</v>
+        <v>326</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L3">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M3">
+        <v>-30</v>
+      </c>
+      <c r="N3">
         <v>30</v>
       </c>
     </row>
@@ -3914,19 +3894,19 @@
         <v>3</v>
       </c>
       <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4">
         <v>4</v>
       </c>
-      <c r="C4">
+      <c r="D4">
         <v>1.12E-2</v>
       </c>
-      <c r="D4">
+      <c r="E4">
         <v>3.6600000000000001E-2</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <v>3.7999999999999999E-2</v>
-      </c>
-      <c r="F4">
-        <v>767</v>
       </c>
       <c r="G4">
         <v>767</v>
@@ -3935,18 +3915,21 @@
         <v>767</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>767</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L4">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M4">
+        <v>-30</v>
+      </c>
+      <c r="N4">
         <v>30</v>
       </c>
     </row>
@@ -3955,19 +3938,19 @@
         <v>4</v>
       </c>
       <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="C5">
         <v>5</v>
       </c>
-      <c r="C5">
+      <c r="D5">
         <v>6.25E-2</v>
       </c>
-      <c r="D5">
+      <c r="E5">
         <v>0.13200000000000001</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <v>2.58E-2</v>
-      </c>
-      <c r="F5">
-        <v>201</v>
       </c>
       <c r="G5">
         <v>201</v>
@@ -3976,39 +3959,42 @@
         <v>201</v>
       </c>
       <c r="I5">
-        <v>0</v>
+        <v>201</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L5">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M5">
+        <v>-30</v>
+      </c>
+      <c r="N5">
         <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
         <v>4</v>
       </c>
-      <c r="B6">
+      <c r="C6">
         <v>6</v>
       </c>
-      <c r="C6">
+      <c r="D6">
         <v>4.2999999999999997E-2</v>
       </c>
-      <c r="D6">
+      <c r="E6">
         <v>0.14799999999999999</v>
       </c>
-      <c r="E6">
+      <c r="F6">
         <v>3.4799999999999998E-2</v>
-      </c>
-      <c r="F6">
-        <v>191</v>
       </c>
       <c r="G6">
         <v>191</v>
@@ -4017,18 +4003,21 @@
         <v>191</v>
       </c>
       <c r="I6">
-        <v>0</v>
+        <v>191</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L6">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M6">
+        <v>-30</v>
+      </c>
+      <c r="N6">
         <v>30</v>
       </c>
     </row>
@@ -4037,19 +4026,19 @@
         <v>6</v>
       </c>
       <c r="B7">
+        <v>6</v>
+      </c>
+      <c r="C7">
         <v>7</v>
       </c>
-      <c r="C7">
+      <c r="D7">
         <v>0.02</v>
       </c>
-      <c r="D7">
+      <c r="E7">
         <v>0.10199999999999999</v>
       </c>
-      <c r="E7">
+      <c r="F7">
         <v>2.76E-2</v>
-      </c>
-      <c r="F7">
-        <v>283</v>
       </c>
       <c r="G7">
         <v>283</v>
@@ -4058,39 +4047,42 @@
         <v>283</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <v>283</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L7">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M7">
+        <v>-30</v>
+      </c>
+      <c r="N7">
         <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
         <v>6</v>
       </c>
-      <c r="B8">
+      <c r="C8">
         <v>8</v>
       </c>
-      <c r="C8">
+      <c r="D8">
         <v>3.39E-2</v>
       </c>
-      <c r="D8">
+      <c r="E8">
         <v>0.17299999999999999</v>
       </c>
-      <c r="E8">
+      <c r="F8">
         <v>4.7E-2</v>
-      </c>
-      <c r="F8">
-        <v>167</v>
       </c>
       <c r="G8">
         <v>167</v>
@@ -4099,18 +4091,21 @@
         <v>167</v>
       </c>
       <c r="I8">
-        <v>0</v>
+        <v>167</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L8">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M8">
+        <v>-30</v>
+      </c>
+      <c r="N8">
         <v>30</v>
       </c>
     </row>
@@ -4119,19 +4114,19 @@
         <v>8</v>
       </c>
       <c r="B9">
+        <v>8</v>
+      </c>
+      <c r="C9">
         <v>9</v>
       </c>
-      <c r="C9">
+      <c r="D9">
         <v>9.9000000000000008E-3</v>
       </c>
-      <c r="D9">
+      <c r="E9">
         <v>5.0500000000000003E-2</v>
       </c>
-      <c r="E9">
+      <c r="F9">
         <v>5.4800000000000001E-2</v>
-      </c>
-      <c r="F9">
-        <v>570</v>
       </c>
       <c r="G9">
         <v>570</v>
@@ -4140,18 +4135,21 @@
         <v>570</v>
       </c>
       <c r="I9">
-        <v>0</v>
+        <v>570</v>
       </c>
       <c r="J9">
         <v>0</v>
       </c>
       <c r="K9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L9">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M9">
+        <v>-30</v>
+      </c>
+      <c r="N9">
         <v>30</v>
       </c>
     </row>
@@ -4160,19 +4158,19 @@
         <v>9</v>
       </c>
       <c r="B10">
+        <v>9</v>
+      </c>
+      <c r="C10">
         <v>10</v>
       </c>
-      <c r="C10">
+      <c r="D10">
         <v>3.6900000000000002E-2</v>
       </c>
-      <c r="D10">
+      <c r="E10">
         <v>0.16789999999999999</v>
       </c>
-      <c r="E10">
+      <c r="F10">
         <v>4.3999999999999997E-2</v>
-      </c>
-      <c r="F10">
-        <v>171</v>
       </c>
       <c r="G10">
         <v>171</v>
@@ -4181,39 +4179,42 @@
         <v>171</v>
       </c>
       <c r="I10">
-        <v>0</v>
+        <v>171</v>
       </c>
       <c r="J10">
         <v>0</v>
       </c>
       <c r="K10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L10">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M10">
+        <v>-30</v>
+      </c>
+      <c r="N10">
         <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
         <v>9</v>
       </c>
-      <c r="B11">
+      <c r="C11">
         <v>11</v>
       </c>
-      <c r="C11">
+      <c r="D11">
         <v>2.58E-2</v>
       </c>
-      <c r="D11">
+      <c r="E11">
         <v>8.48E-2</v>
       </c>
-      <c r="E11">
+      <c r="F11">
         <v>2.18E-2</v>
-      </c>
-      <c r="F11">
-        <v>331</v>
       </c>
       <c r="G11">
         <v>331</v>
@@ -4222,39 +4223,42 @@
         <v>331</v>
       </c>
       <c r="I11">
-        <v>0</v>
+        <v>331</v>
       </c>
       <c r="J11">
         <v>0</v>
       </c>
       <c r="K11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L11">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M11">
+        <v>-30</v>
+      </c>
+      <c r="N11">
         <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12">
         <v>9</v>
       </c>
-      <c r="B12">
+      <c r="C12">
         <v>12</v>
       </c>
-      <c r="C12">
+      <c r="D12">
         <v>6.4799999999999996E-2</v>
       </c>
-      <c r="D12">
+      <c r="E12">
         <v>0.29499999999999998</v>
       </c>
-      <c r="E12">
+      <c r="F12">
         <v>7.7200000000000005E-2</v>
-      </c>
-      <c r="F12">
-        <v>98</v>
       </c>
       <c r="G12">
         <v>98</v>
@@ -4263,39 +4267,42 @@
         <v>98</v>
       </c>
       <c r="I12">
-        <v>0</v>
+        <v>98</v>
       </c>
       <c r="J12">
         <v>0</v>
       </c>
       <c r="K12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L12">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M12">
+        <v>-30</v>
+      </c>
+      <c r="N12">
         <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13">
         <v>9</v>
       </c>
-      <c r="B13">
+      <c r="C13">
         <v>13</v>
       </c>
-      <c r="C13">
+      <c r="D13">
         <v>4.8099999999999997E-2</v>
       </c>
-      <c r="D13">
+      <c r="E13">
         <v>0.158</v>
       </c>
-      <c r="E13">
+      <c r="F13">
         <v>4.0599999999999997E-2</v>
-      </c>
-      <c r="F13">
-        <v>178</v>
       </c>
       <c r="G13">
         <v>178</v>
@@ -4304,18 +4311,21 @@
         <v>178</v>
       </c>
       <c r="I13">
-        <v>0</v>
+        <v>178</v>
       </c>
       <c r="J13">
         <v>0</v>
       </c>
       <c r="K13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L13">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M13">
+        <v>-30</v>
+      </c>
+      <c r="N13">
         <v>30</v>
       </c>
     </row>
@@ -4324,19 +4334,19 @@
         <v>13</v>
       </c>
       <c r="B14">
+        <v>13</v>
+      </c>
+      <c r="C14">
         <v>14</v>
       </c>
-      <c r="C14">
+      <c r="D14">
         <v>1.32E-2</v>
       </c>
-      <c r="D14">
+      <c r="E14">
         <v>4.3400000000000001E-2</v>
       </c>
-      <c r="E14">
+      <c r="F14">
         <v>1.0999999999999999E-2</v>
-      </c>
-      <c r="F14">
-        <v>647</v>
       </c>
       <c r="G14">
         <v>647</v>
@@ -4345,39 +4355,42 @@
         <v>647</v>
       </c>
       <c r="I14">
-        <v>0</v>
+        <v>647</v>
       </c>
       <c r="J14">
         <v>0</v>
       </c>
       <c r="K14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L14">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M14">
+        <v>-30</v>
+      </c>
+      <c r="N14">
         <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15">
         <v>13</v>
       </c>
-      <c r="B15">
+      <c r="C15">
         <v>15</v>
       </c>
-      <c r="C15">
+      <c r="D15">
         <v>2.69E-2</v>
       </c>
-      <c r="D15">
+      <c r="E15">
         <v>8.6900000000000005E-2</v>
       </c>
-      <c r="E15">
+      <c r="F15">
         <v>2.3E-2</v>
-      </c>
-      <c r="F15">
-        <v>323</v>
       </c>
       <c r="G15">
         <v>323</v>
@@ -4386,39 +4399,42 @@
         <v>323</v>
       </c>
       <c r="I15">
-        <v>0</v>
+        <v>323</v>
       </c>
       <c r="J15">
         <v>0</v>
       </c>
       <c r="K15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L15">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M15">
+        <v>-30</v>
+      </c>
+      <c r="N15">
         <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="B16">
+        <v>1</v>
+      </c>
+      <c r="C16">
         <v>15</v>
       </c>
-      <c r="C16">
+      <c r="D16">
         <v>1.78E-2</v>
       </c>
-      <c r="D16">
+      <c r="E16">
         <v>9.0999999999999998E-2</v>
       </c>
-      <c r="E16">
+      <c r="F16">
         <v>9.8799999999999999E-2</v>
-      </c>
-      <c r="F16">
-        <v>317</v>
       </c>
       <c r="G16">
         <v>317</v>
@@ -4427,39 +4443,42 @@
         <v>317</v>
       </c>
       <c r="I16">
-        <v>0</v>
+        <v>317</v>
       </c>
       <c r="J16">
         <v>0</v>
       </c>
       <c r="K16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L16">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M16">
+        <v>-30</v>
+      </c>
+      <c r="N16">
         <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="B17">
+        <v>1</v>
+      </c>
+      <c r="C17">
         <v>16</v>
       </c>
-      <c r="C17">
+      <c r="D17">
         <v>4.5400000000000003E-2</v>
       </c>
-      <c r="D17">
+      <c r="E17">
         <v>0.20599999999999999</v>
       </c>
-      <c r="E17">
+      <c r="F17">
         <v>5.4600000000000003E-2</v>
-      </c>
-      <c r="F17">
-        <v>140</v>
       </c>
       <c r="G17">
         <v>140</v>
@@ -4468,39 +4487,42 @@
         <v>140</v>
       </c>
       <c r="I17">
-        <v>0</v>
+        <v>140</v>
       </c>
       <c r="J17">
         <v>0</v>
       </c>
       <c r="K17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L17">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M17">
+        <v>-30</v>
+      </c>
+      <c r="N17">
         <v>30</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="B18">
+        <v>1</v>
+      </c>
+      <c r="C18">
         <v>17</v>
       </c>
-      <c r="C18">
+      <c r="D18">
         <v>2.3800000000000002E-2</v>
       </c>
-      <c r="D18">
+      <c r="E18">
         <v>0.108</v>
       </c>
-      <c r="E18">
+      <c r="F18">
         <v>2.86E-2</v>
-      </c>
-      <c r="F18">
-        <v>266</v>
       </c>
       <c r="G18">
         <v>266</v>
@@ -4509,39 +4531,42 @@
         <v>266</v>
       </c>
       <c r="I18">
-        <v>0</v>
+        <v>266</v>
       </c>
       <c r="J18">
         <v>0</v>
       </c>
       <c r="K18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L18">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M18">
+        <v>-30</v>
+      </c>
+      <c r="N18">
         <v>30</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19">
         <v>3</v>
       </c>
-      <c r="B19">
+      <c r="C19">
         <v>15</v>
       </c>
-      <c r="C19">
+      <c r="D19">
         <v>1.6199999999999999E-2</v>
       </c>
-      <c r="D19">
+      <c r="E19">
         <v>5.2999999999999999E-2</v>
       </c>
-      <c r="E19">
+      <c r="F19">
         <v>5.4399999999999997E-2</v>
-      </c>
-      <c r="F19">
-        <v>530</v>
       </c>
       <c r="G19">
         <v>530</v>
@@ -4550,127 +4575,130 @@
         <v>530</v>
       </c>
       <c r="I19">
-        <v>0</v>
+        <v>530</v>
       </c>
       <c r="J19">
         <v>0</v>
       </c>
       <c r="K19">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L19">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M19">
+        <v>-30</v>
+      </c>
+      <c r="N19">
         <v>30</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A20" s="3">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2">
         <v>4</v>
       </c>
-      <c r="B20" s="3">
+      <c r="C20" s="2">
         <v>18</v>
       </c>
-      <c r="C20" s="3">
-        <v>0</v>
-      </c>
-      <c r="D20" s="3">
+      <c r="D20" s="2">
+        <v>0</v>
+      </c>
+      <c r="E20" s="2">
         <v>0.55500000000000005</v>
       </c>
-      <c r="E20" s="3">
-        <v>0</v>
-      </c>
-      <c r="F20" s="3">
+      <c r="F20" s="2">
+        <v>0</v>
+      </c>
+      <c r="G20" s="2">
         <v>53</v>
       </c>
-      <c r="G20" s="3">
+      <c r="H20" s="2">
         <v>53</v>
       </c>
-      <c r="H20" s="3">
+      <c r="I20" s="2">
         <v>53</v>
       </c>
-      <c r="I20" s="3">
+      <c r="J20" s="2">
         <v>0.97</v>
       </c>
-      <c r="J20" s="3">
-        <v>0</v>
-      </c>
-      <c r="K20" s="3">
-        <v>1</v>
-      </c>
-      <c r="L20" s="3">
-        <v>-30</v>
-      </c>
-      <c r="M20" s="3">
-        <v>30</v>
-      </c>
-      <c r="N20">
-        <v>1</v>
+      <c r="K20" s="2">
+        <v>0</v>
+      </c>
+      <c r="L20" s="2">
+        <v>1</v>
+      </c>
+      <c r="M20" s="2">
+        <v>-30</v>
+      </c>
+      <c r="N20" s="2">
+        <v>30</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A21" s="3">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2">
         <v>4</v>
       </c>
-      <c r="B21" s="3">
+      <c r="C21" s="2">
         <v>18</v>
       </c>
-      <c r="C21" s="3">
-        <v>0</v>
-      </c>
-      <c r="D21" s="3">
+      <c r="D21" s="2">
+        <v>0</v>
+      </c>
+      <c r="E21" s="2">
         <v>0.43</v>
       </c>
-      <c r="E21" s="3">
-        <v>0</v>
-      </c>
-      <c r="F21" s="3">
+      <c r="F21" s="2">
+        <v>0</v>
+      </c>
+      <c r="G21" s="2">
         <v>69</v>
       </c>
-      <c r="G21" s="3">
+      <c r="H21" s="2">
         <v>69</v>
       </c>
-      <c r="H21" s="3">
+      <c r="I21" s="2">
         <v>69</v>
       </c>
-      <c r="I21" s="3">
+      <c r="J21" s="2">
         <v>0.97799999999999998</v>
       </c>
-      <c r="J21" s="3">
-        <v>0</v>
-      </c>
-      <c r="K21" s="3">
-        <v>1</v>
-      </c>
-      <c r="L21" s="3">
-        <v>-30</v>
-      </c>
-      <c r="M21" s="3">
-        <v>30</v>
-      </c>
-      <c r="N21">
-        <v>1</v>
+      <c r="K21" s="2">
+        <v>0</v>
+      </c>
+      <c r="L21" s="2">
+        <v>1</v>
+      </c>
+      <c r="M21" s="2">
+        <v>-30</v>
+      </c>
+      <c r="N21" s="2">
+        <v>30</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22">
         <v>5</v>
       </c>
-      <c r="B22">
+      <c r="C22">
         <v>6</v>
       </c>
-      <c r="C22">
+      <c r="D22">
         <v>3.0200000000000001E-2</v>
       </c>
-      <c r="D22">
+      <c r="E22">
         <v>6.4100000000000004E-2</v>
       </c>
-      <c r="E22">
+      <c r="F22">
         <v>1.24E-2</v>
-      </c>
-      <c r="F22">
-        <v>414</v>
       </c>
       <c r="G22">
         <v>414</v>
@@ -4679,39 +4707,42 @@
         <v>414</v>
       </c>
       <c r="I22">
-        <v>0</v>
+        <v>414</v>
       </c>
       <c r="J22">
         <v>0</v>
       </c>
       <c r="K22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L22">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M22">
+        <v>-30</v>
+      </c>
+      <c r="N22">
         <v>30</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23">
         <v>7</v>
       </c>
-      <c r="B23">
+      <c r="C23">
         <v>8</v>
       </c>
-      <c r="C23">
+      <c r="D23">
         <v>1.3899999999999999E-2</v>
       </c>
-      <c r="D23">
+      <c r="E23">
         <v>7.1199999999999999E-2</v>
       </c>
-      <c r="E23">
+      <c r="F23">
         <v>1.9400000000000001E-2</v>
-      </c>
-      <c r="F23">
-        <v>405</v>
       </c>
       <c r="G23">
         <v>405</v>
@@ -4720,39 +4751,42 @@
         <v>405</v>
       </c>
       <c r="I23">
-        <v>0</v>
+        <v>405</v>
       </c>
       <c r="J23">
         <v>0</v>
       </c>
       <c r="K23">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L23">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M23">
+        <v>-30</v>
+      </c>
+      <c r="N23">
         <v>30</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24">
         <v>10</v>
       </c>
-      <c r="B24">
+      <c r="C24">
         <v>12</v>
       </c>
-      <c r="C24">
+      <c r="D24">
         <v>2.7699999999999999E-2</v>
       </c>
-      <c r="D24">
+      <c r="E24">
         <v>0.12620000000000001</v>
       </c>
-      <c r="E24">
+      <c r="F24">
         <v>3.2800000000000003E-2</v>
-      </c>
-      <c r="F24">
-        <v>228</v>
       </c>
       <c r="G24">
         <v>228</v>
@@ -4761,39 +4795,42 @@
         <v>228</v>
       </c>
       <c r="I24">
-        <v>0</v>
+        <v>228</v>
       </c>
       <c r="J24">
         <v>0</v>
       </c>
       <c r="K24">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L24">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M24">
+        <v>-30</v>
+      </c>
+      <c r="N24">
         <v>30</v>
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25">
         <v>11</v>
       </c>
-      <c r="B25">
+      <c r="C25">
         <v>13</v>
       </c>
-      <c r="C25">
+      <c r="D25">
         <v>2.23E-2</v>
       </c>
-      <c r="D25">
+      <c r="E25">
         <v>7.3200000000000001E-2</v>
       </c>
-      <c r="E25">
+      <c r="F25">
         <v>1.8800000000000001E-2</v>
-      </c>
-      <c r="F25">
-        <v>384</v>
       </c>
       <c r="G25">
         <v>384</v>
@@ -4802,39 +4839,42 @@
         <v>384</v>
       </c>
       <c r="I25">
-        <v>0</v>
+        <v>384</v>
       </c>
       <c r="J25">
         <v>0</v>
       </c>
       <c r="K25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L25">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M25">
+        <v>-30</v>
+      </c>
+      <c r="N25">
         <v>30</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26">
         <v>12</v>
       </c>
-      <c r="B26">
+      <c r="C26">
         <v>13</v>
       </c>
-      <c r="C26">
+      <c r="D26">
         <v>1.78E-2</v>
       </c>
-      <c r="D26">
+      <c r="E26">
         <v>5.8000000000000003E-2</v>
       </c>
-      <c r="E26">
+      <c r="F26">
         <v>6.0400000000000002E-2</v>
-      </c>
-      <c r="F26">
-        <v>484</v>
       </c>
       <c r="G26">
         <v>484</v>
@@ -4843,39 +4883,42 @@
         <v>484</v>
       </c>
       <c r="I26">
-        <v>0</v>
+        <v>484</v>
       </c>
       <c r="J26">
         <v>0</v>
       </c>
       <c r="K26">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L26">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M26">
+        <v>-30</v>
+      </c>
+      <c r="N26">
         <v>30</v>
       </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27">
         <v>12</v>
       </c>
-      <c r="B27">
+      <c r="C27">
         <v>16</v>
       </c>
-      <c r="C27">
+      <c r="D27">
         <v>1.7999999999999999E-2</v>
       </c>
-      <c r="D27">
+      <c r="E27">
         <v>8.1299999999999997E-2</v>
       </c>
-      <c r="E27">
+      <c r="F27">
         <v>2.1600000000000001E-2</v>
-      </c>
-      <c r="F27">
-        <v>353</v>
       </c>
       <c r="G27">
         <v>353</v>
@@ -4884,39 +4927,42 @@
         <v>353</v>
       </c>
       <c r="I27">
-        <v>0</v>
+        <v>353</v>
       </c>
       <c r="J27">
         <v>0</v>
       </c>
       <c r="K27">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L27">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M27">
+        <v>-30</v>
+      </c>
+      <c r="N27">
         <v>30</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28">
         <v>12</v>
       </c>
-      <c r="B28">
+      <c r="C28">
         <v>17</v>
       </c>
-      <c r="C28">
+      <c r="D28">
         <v>3.9699999999999999E-2</v>
       </c>
-      <c r="D28">
+      <c r="E28">
         <v>0.17899999999999999</v>
       </c>
-      <c r="E28">
+      <c r="F28">
         <v>4.7600000000000003E-2</v>
-      </c>
-      <c r="F28">
-        <v>160</v>
       </c>
       <c r="G28">
         <v>160</v>
@@ -4925,39 +4971,42 @@
         <v>160</v>
       </c>
       <c r="I28">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="J28">
         <v>0</v>
       </c>
       <c r="K28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L28">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M28">
+        <v>-30</v>
+      </c>
+      <c r="N28">
         <v>30</v>
       </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29">
         <v>14</v>
       </c>
-      <c r="B29">
+      <c r="C29">
         <v>15</v>
       </c>
-      <c r="C29">
+      <c r="D29">
         <v>1.7100000000000001E-2</v>
       </c>
-      <c r="D29">
+      <c r="E29">
         <v>5.4699999999999999E-2</v>
       </c>
-      <c r="E29">
+      <c r="F29">
         <v>1.4800000000000001E-2</v>
-      </c>
-      <c r="F29">
-        <v>512</v>
       </c>
       <c r="G29">
         <v>512</v>
@@ -4966,39 +5015,42 @@
         <v>512</v>
       </c>
       <c r="I29">
-        <v>0</v>
+        <v>512</v>
       </c>
       <c r="J29">
         <v>0</v>
       </c>
       <c r="K29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L29">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M29">
+        <v>-30</v>
+      </c>
+      <c r="N29">
         <v>30</v>
       </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30">
         <v>18</v>
       </c>
-      <c r="B30">
+      <c r="C30">
         <v>19</v>
       </c>
-      <c r="C30">
+      <c r="D30">
         <v>0.46100000000000002</v>
       </c>
-      <c r="D30">
+      <c r="E30">
         <v>0.68500000000000005</v>
       </c>
-      <c r="E30">
-        <v>0</v>
-      </c>
       <c r="F30">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="G30">
         <v>36</v>
@@ -5007,39 +5059,42 @@
         <v>36</v>
       </c>
       <c r="I30">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="J30">
         <v>0</v>
       </c>
       <c r="K30">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L30">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M30">
+        <v>-30</v>
+      </c>
+      <c r="N30">
         <v>30</v>
       </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31">
         <v>19</v>
       </c>
-      <c r="B31">
+      <c r="C31">
         <v>20</v>
       </c>
-      <c r="C31">
+      <c r="D31">
         <v>0.28299999999999997</v>
       </c>
-      <c r="D31">
+      <c r="E31">
         <v>0.434</v>
       </c>
-      <c r="E31">
-        <v>0</v>
-      </c>
       <c r="F31">
-        <v>57</v>
+        <v>0</v>
       </c>
       <c r="G31">
         <v>57</v>
@@ -5048,39 +5103,42 @@
         <v>57</v>
       </c>
       <c r="I31">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="J31">
         <v>0</v>
       </c>
       <c r="K31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L31">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M31">
+        <v>-30</v>
+      </c>
+      <c r="N31">
         <v>30</v>
       </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32">
         <v>21</v>
       </c>
-      <c r="B32">
+      <c r="C32">
         <v>20</v>
       </c>
-      <c r="C32">
-        <v>0</v>
-      </c>
       <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32">
         <v>0.77669999999999995</v>
       </c>
-      <c r="E32">
-        <v>0</v>
-      </c>
       <c r="F32">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="G32">
         <v>38</v>
@@ -5089,39 +5147,42 @@
         <v>38</v>
       </c>
       <c r="I32">
+        <v>38</v>
+      </c>
+      <c r="J32">
         <v>1.0429999999999999</v>
       </c>
-      <c r="J32">
-        <v>0</v>
-      </c>
       <c r="K32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L32">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M32">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N32">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33">
         <v>21</v>
       </c>
-      <c r="B33">
+      <c r="C33">
         <v>22</v>
       </c>
-      <c r="C33">
+      <c r="D33">
         <v>7.3599999999999999E-2</v>
       </c>
-      <c r="D33">
+      <c r="E33">
         <v>0.11700000000000001</v>
       </c>
-      <c r="E33">
-        <v>0</v>
-      </c>
       <c r="F33">
-        <v>213</v>
+        <v>0</v>
       </c>
       <c r="G33">
         <v>213</v>
@@ -5130,39 +5191,42 @@
         <v>213</v>
       </c>
       <c r="I33">
-        <v>0</v>
+        <v>213</v>
       </c>
       <c r="J33">
         <v>0</v>
       </c>
       <c r="K33">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L33">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M33">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N33">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34">
         <v>22</v>
       </c>
-      <c r="B34">
+      <c r="C34">
         <v>23</v>
       </c>
-      <c r="C34">
+      <c r="D34">
         <v>9.9000000000000008E-3</v>
       </c>
-      <c r="D34">
+      <c r="E34">
         <v>1.52E-2</v>
       </c>
-      <c r="E34">
-        <v>0</v>
-      </c>
       <c r="F34">
-        <v>1617</v>
+        <v>0</v>
       </c>
       <c r="G34">
         <v>1617</v>
@@ -5171,39 +5235,42 @@
         <v>1617</v>
       </c>
       <c r="I34">
-        <v>0</v>
+        <v>1617</v>
       </c>
       <c r="J34">
         <v>0</v>
       </c>
       <c r="K34">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L34">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M34">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N34">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35">
         <v>23</v>
       </c>
-      <c r="B35">
+      <c r="C35">
         <v>24</v>
       </c>
-      <c r="C35">
+      <c r="D35">
         <v>0.16600000000000001</v>
       </c>
-      <c r="D35">
+      <c r="E35">
         <v>0.25600000000000001</v>
       </c>
-      <c r="E35">
+      <c r="F35">
         <v>8.3999999999999995E-3</v>
-      </c>
-      <c r="F35">
-        <v>97</v>
       </c>
       <c r="G35">
         <v>97</v>
@@ -5212,39 +5279,42 @@
         <v>97</v>
       </c>
       <c r="I35">
-        <v>0</v>
+        <v>97</v>
       </c>
       <c r="J35">
         <v>0</v>
       </c>
       <c r="K35">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L35">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M35">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N35">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36">
         <v>24</v>
       </c>
-      <c r="B36">
+      <c r="C36">
         <v>25</v>
       </c>
-      <c r="C36">
-        <v>0</v>
-      </c>
       <c r="D36">
+        <v>0</v>
+      </c>
+      <c r="E36">
         <v>1.1819999999999999</v>
       </c>
-      <c r="E36">
-        <v>0</v>
-      </c>
       <c r="F36">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="G36">
         <v>25</v>
@@ -5253,39 +5323,42 @@
         <v>25</v>
       </c>
       <c r="I36">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="J36">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K36">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L36">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M36">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N36">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37">
         <v>24</v>
       </c>
-      <c r="B37">
+      <c r="C37">
         <v>25</v>
       </c>
-      <c r="C37">
-        <v>0</v>
-      </c>
       <c r="D37">
+        <v>0</v>
+      </c>
+      <c r="E37">
         <v>1.23</v>
       </c>
-      <c r="E37">
-        <v>0</v>
-      </c>
       <c r="F37">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="G37">
         <v>24</v>
@@ -5294,39 +5367,42 @@
         <v>24</v>
       </c>
       <c r="I37">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="J37">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K37">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L37">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M37">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N37">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38">
         <v>24</v>
       </c>
-      <c r="B38">
+      <c r="C38">
         <v>26</v>
       </c>
-      <c r="C38">
-        <v>0</v>
-      </c>
       <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38">
         <v>4.7300000000000002E-2</v>
       </c>
-      <c r="E38">
-        <v>0</v>
-      </c>
       <c r="F38">
-        <v>621</v>
+        <v>0</v>
       </c>
       <c r="G38">
         <v>621</v>
@@ -5335,39 +5411,42 @@
         <v>621</v>
       </c>
       <c r="I38">
+        <v>621</v>
+      </c>
+      <c r="J38">
         <v>1.0429999999999999</v>
       </c>
-      <c r="J38">
-        <v>0</v>
-      </c>
       <c r="K38">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L38">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M38">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N38">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39">
         <v>26</v>
       </c>
-      <c r="B39">
+      <c r="C39">
         <v>27</v>
       </c>
-      <c r="C39">
+      <c r="D39">
         <v>0.16500000000000001</v>
       </c>
-      <c r="D39">
+      <c r="E39">
         <v>0.254</v>
       </c>
-      <c r="E39">
-        <v>0</v>
-      </c>
       <c r="F39">
-        <v>97</v>
+        <v>0</v>
       </c>
       <c r="G39">
         <v>97</v>
@@ -5376,39 +5455,42 @@
         <v>97</v>
       </c>
       <c r="I39">
-        <v>0</v>
+        <v>97</v>
       </c>
       <c r="J39">
         <v>0</v>
       </c>
       <c r="K39">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L39">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M39">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N39">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40">
         <v>27</v>
       </c>
-      <c r="B40">
+      <c r="C40">
         <v>28</v>
       </c>
-      <c r="C40">
+      <c r="D40">
         <v>6.1800000000000001E-2</v>
       </c>
-      <c r="D40">
+      <c r="E40">
         <v>9.5399999999999999E-2</v>
       </c>
-      <c r="E40">
-        <v>0</v>
-      </c>
       <c r="F40">
-        <v>259</v>
+        <v>0</v>
       </c>
       <c r="G40">
         <v>259</v>
@@ -5417,39 +5499,42 @@
         <v>259</v>
       </c>
       <c r="I40">
-        <v>0</v>
+        <v>259</v>
       </c>
       <c r="J40">
         <v>0</v>
       </c>
       <c r="K40">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L40">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M40">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N40">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41">
         <v>28</v>
       </c>
-      <c r="B41">
+      <c r="C41">
         <v>29</v>
       </c>
-      <c r="C41">
+      <c r="D41">
         <v>4.1799999999999997E-2</v>
       </c>
-      <c r="D41">
+      <c r="E41">
         <v>5.8700000000000002E-2</v>
       </c>
-      <c r="E41">
-        <v>0</v>
-      </c>
       <c r="F41">
-        <v>408</v>
+        <v>0</v>
       </c>
       <c r="G41">
         <v>408</v>
@@ -5458,39 +5543,42 @@
         <v>408</v>
       </c>
       <c r="I41">
-        <v>0</v>
+        <v>408</v>
       </c>
       <c r="J41">
         <v>0</v>
       </c>
       <c r="K41">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L41">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M41">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N41">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42">
         <v>7</v>
       </c>
-      <c r="B42">
+      <c r="C42">
         <v>29</v>
       </c>
-      <c r="C42">
-        <v>0</v>
-      </c>
       <c r="D42">
+        <v>0</v>
+      </c>
+      <c r="E42">
         <v>6.4799999999999996E-2</v>
       </c>
-      <c r="E42">
-        <v>0</v>
-      </c>
       <c r="F42">
-        <v>453</v>
+        <v>0</v>
       </c>
       <c r="G42">
         <v>453</v>
@@ -5499,39 +5587,42 @@
         <v>453</v>
       </c>
       <c r="I42">
+        <v>453</v>
+      </c>
+      <c r="J42">
         <v>0.96699999999999997</v>
       </c>
-      <c r="J42">
-        <v>0</v>
-      </c>
       <c r="K42">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L42">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M42">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N42">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43">
         <v>25</v>
       </c>
-      <c r="B43">
-        <v>30</v>
-      </c>
       <c r="C43">
+        <v>30</v>
+      </c>
+      <c r="D43">
         <v>0.13500000000000001</v>
       </c>
-      <c r="D43">
+      <c r="E43">
         <v>0.20200000000000001</v>
       </c>
-      <c r="E43">
-        <v>0</v>
-      </c>
       <c r="F43">
-        <v>121</v>
+        <v>0</v>
       </c>
       <c r="G43">
         <v>121</v>
@@ -5540,39 +5631,42 @@
         <v>121</v>
       </c>
       <c r="I43">
-        <v>0</v>
+        <v>121</v>
       </c>
       <c r="J43">
         <v>0</v>
       </c>
       <c r="K43">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L43">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M43">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N43">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A44">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="B44">
+        <v>30</v>
+      </c>
+      <c r="C44">
         <v>31</v>
       </c>
-      <c r="C44">
+      <c r="D44">
         <v>0.32600000000000001</v>
       </c>
-      <c r="D44">
+      <c r="E44">
         <v>0.497</v>
       </c>
-      <c r="E44">
-        <v>0</v>
-      </c>
       <c r="F44">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="G44">
         <v>50</v>
@@ -5581,39 +5675,42 @@
         <v>50</v>
       </c>
       <c r="I44">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="J44">
         <v>0</v>
       </c>
       <c r="K44">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L44">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M44">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N44">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45">
         <v>31</v>
       </c>
-      <c r="B45">
+      <c r="C45">
         <v>32</v>
       </c>
-      <c r="C45">
+      <c r="D45">
         <v>0.50700000000000001</v>
       </c>
-      <c r="D45">
+      <c r="E45">
         <v>0.755</v>
       </c>
-      <c r="E45">
-        <v>0</v>
-      </c>
       <c r="F45">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="G45">
         <v>33</v>
@@ -5622,39 +5719,42 @@
         <v>33</v>
       </c>
       <c r="I45">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="J45">
         <v>0</v>
       </c>
       <c r="K45">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L45">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M45">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N45">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46">
         <v>32</v>
       </c>
-      <c r="B46">
+      <c r="C46">
         <v>33</v>
       </c>
-      <c r="C46">
+      <c r="D46">
         <v>3.9199999999999999E-2</v>
       </c>
-      <c r="D46">
+      <c r="E46">
         <v>3.5999999999999997E-2</v>
       </c>
-      <c r="E46">
-        <v>0</v>
-      </c>
       <c r="F46">
-        <v>552</v>
+        <v>0</v>
       </c>
       <c r="G46">
         <v>552</v>
@@ -5663,39 +5763,42 @@
         <v>552</v>
       </c>
       <c r="I46">
-        <v>0</v>
+        <v>552</v>
       </c>
       <c r="J46">
         <v>0</v>
       </c>
       <c r="K46">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L46">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M46">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N46">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47">
         <v>34</v>
       </c>
-      <c r="B47">
+      <c r="C47">
         <v>32</v>
       </c>
-      <c r="C47">
-        <v>0</v>
-      </c>
       <c r="D47">
+        <v>0</v>
+      </c>
+      <c r="E47">
         <v>0.95299999999999996</v>
       </c>
-      <c r="E47">
-        <v>0</v>
-      </c>
       <c r="F47">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="G47">
         <v>31</v>
@@ -5704,39 +5807,42 @@
         <v>31</v>
       </c>
       <c r="I47">
+        <v>31</v>
+      </c>
+      <c r="J47">
         <v>0.97499999999999998</v>
       </c>
-      <c r="J47">
-        <v>0</v>
-      </c>
       <c r="K47">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L47">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M47">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N47">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48">
         <v>34</v>
       </c>
-      <c r="B48">
+      <c r="C48">
         <v>35</v>
       </c>
-      <c r="C48">
+      <c r="D48">
         <v>5.1999999999999998E-2</v>
       </c>
-      <c r="D48">
+      <c r="E48">
         <v>7.8E-2</v>
       </c>
-      <c r="E48">
+      <c r="F48">
         <v>3.2000000000000002E-3</v>
-      </c>
-      <c r="F48">
-        <v>313</v>
       </c>
       <c r="G48">
         <v>313</v>
@@ -5745,39 +5851,42 @@
         <v>313</v>
       </c>
       <c r="I48">
-        <v>0</v>
+        <v>313</v>
       </c>
       <c r="J48">
         <v>0</v>
       </c>
       <c r="K48">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L48">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M48">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N48">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49">
         <v>35</v>
       </c>
-      <c r="B49">
+      <c r="C49">
         <v>36</v>
       </c>
-      <c r="C49">
+      <c r="D49">
         <v>4.2999999999999997E-2</v>
       </c>
-      <c r="D49">
+      <c r="E49">
         <v>5.3699999999999998E-2</v>
       </c>
-      <c r="E49">
+      <c r="F49">
         <v>1.6000000000000001E-3</v>
-      </c>
-      <c r="F49">
-        <v>427</v>
       </c>
       <c r="G49">
         <v>427</v>
@@ -5786,39 +5895,42 @@
         <v>427</v>
       </c>
       <c r="I49">
-        <v>0</v>
+        <v>427</v>
       </c>
       <c r="J49">
         <v>0</v>
       </c>
       <c r="K49">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L49">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M49">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N49">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50">
         <v>36</v>
       </c>
-      <c r="B50">
+      <c r="C50">
         <v>37</v>
       </c>
-      <c r="C50">
+      <c r="D50">
         <v>2.9000000000000001E-2</v>
       </c>
-      <c r="D50">
+      <c r="E50">
         <v>3.6600000000000001E-2</v>
       </c>
-      <c r="E50">
-        <v>0</v>
-      </c>
       <c r="F50">
-        <v>629</v>
+        <v>0</v>
       </c>
       <c r="G50">
         <v>629</v>
@@ -5827,39 +5939,42 @@
         <v>629</v>
       </c>
       <c r="I50">
-        <v>0</v>
+        <v>629</v>
       </c>
       <c r="J50">
         <v>0</v>
       </c>
       <c r="K50">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L50">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M50">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N50">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51">
         <v>37</v>
       </c>
-      <c r="B51">
+      <c r="C51">
         <v>38</v>
       </c>
-      <c r="C51">
+      <c r="D51">
         <v>6.5100000000000005E-2</v>
       </c>
-      <c r="D51">
+      <c r="E51">
         <v>0.1009</v>
       </c>
-      <c r="E51">
+      <c r="F51">
         <v>2E-3</v>
-      </c>
-      <c r="F51">
-        <v>245</v>
       </c>
       <c r="G51">
         <v>245</v>
@@ -5868,39 +5983,42 @@
         <v>245</v>
       </c>
       <c r="I51">
-        <v>0</v>
+        <v>245</v>
       </c>
       <c r="J51">
         <v>0</v>
       </c>
       <c r="K51">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L51">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M51">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N51">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52">
         <v>37</v>
       </c>
-      <c r="B52">
+      <c r="C52">
         <v>39</v>
       </c>
-      <c r="C52">
+      <c r="D52">
         <v>2.3900000000000001E-2</v>
       </c>
-      <c r="D52">
+      <c r="E52">
         <v>3.7900000000000003E-2</v>
       </c>
-      <c r="E52">
-        <v>0</v>
-      </c>
       <c r="F52">
-        <v>655</v>
+        <v>0</v>
       </c>
       <c r="G52">
         <v>655</v>
@@ -5909,39 +6027,42 @@
         <v>655</v>
       </c>
       <c r="I52">
-        <v>0</v>
+        <v>655</v>
       </c>
       <c r="J52">
         <v>0</v>
       </c>
       <c r="K52">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L52">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M52">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N52">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53">
         <v>36</v>
       </c>
-      <c r="B53">
+      <c r="C53">
         <v>40</v>
       </c>
-      <c r="C53">
+      <c r="D53">
         <v>0.03</v>
       </c>
-      <c r="D53">
+      <c r="E53">
         <v>4.6600000000000003E-2</v>
       </c>
-      <c r="E53">
-        <v>0</v>
-      </c>
       <c r="F53">
-        <v>530</v>
+        <v>0</v>
       </c>
       <c r="G53">
         <v>530</v>
@@ -5950,39 +6071,42 @@
         <v>530</v>
       </c>
       <c r="I53">
-        <v>0</v>
+        <v>530</v>
       </c>
       <c r="J53">
         <v>0</v>
       </c>
       <c r="K53">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L53">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M53">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N53">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54">
         <v>22</v>
       </c>
-      <c r="B54">
+      <c r="C54">
         <v>38</v>
       </c>
-      <c r="C54">
+      <c r="D54">
         <v>1.9199999999999998E-2</v>
       </c>
-      <c r="D54">
+      <c r="E54">
         <v>2.9499999999999998E-2</v>
       </c>
-      <c r="E54">
-        <v>0</v>
-      </c>
       <c r="F54">
-        <v>834</v>
+        <v>0</v>
       </c>
       <c r="G54">
         <v>834</v>
@@ -5991,39 +6115,42 @@
         <v>834</v>
       </c>
       <c r="I54">
-        <v>0</v>
+        <v>834</v>
       </c>
       <c r="J54">
         <v>0</v>
       </c>
       <c r="K54">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L54">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M54">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N54">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55">
         <v>11</v>
       </c>
-      <c r="B55">
+      <c r="C55">
         <v>41</v>
       </c>
-      <c r="C55">
-        <v>0</v>
-      </c>
       <c r="D55">
+        <v>0</v>
+      </c>
+      <c r="E55">
         <v>0.749</v>
       </c>
-      <c r="E55">
-        <v>0</v>
-      </c>
       <c r="F55">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="G55">
         <v>40</v>
@@ -6032,39 +6159,42 @@
         <v>40</v>
       </c>
       <c r="I55">
+        <v>40</v>
+      </c>
+      <c r="J55">
         <v>0.95499999999999996</v>
       </c>
-      <c r="J55">
-        <v>0</v>
-      </c>
       <c r="K55">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L55">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M55">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N55">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56">
         <v>41</v>
       </c>
-      <c r="B56">
+      <c r="C56">
         <v>42</v>
       </c>
-      <c r="C56">
+      <c r="D56">
         <v>0.20699999999999999</v>
       </c>
-      <c r="D56">
+      <c r="E56">
         <v>0.35199999999999998</v>
       </c>
-      <c r="E56">
-        <v>0</v>
-      </c>
       <c r="F56">
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="G56">
         <v>72</v>
@@ -6073,39 +6203,42 @@
         <v>72</v>
       </c>
       <c r="I56">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="J56">
         <v>0</v>
       </c>
       <c r="K56">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L56">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M56">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N56">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57">
         <v>41</v>
       </c>
-      <c r="B57">
+      <c r="C57">
         <v>43</v>
       </c>
-      <c r="C57">
-        <v>0</v>
-      </c>
       <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57">
         <v>0.41199999999999998</v>
       </c>
-      <c r="E57">
-        <v>0</v>
-      </c>
       <c r="F57">
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="G57">
         <v>72</v>
@@ -6114,39 +6247,42 @@
         <v>72</v>
       </c>
       <c r="I57">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="J57">
         <v>0</v>
       </c>
       <c r="K57">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L57">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M57">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N57">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="58" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58">
         <v>38</v>
       </c>
-      <c r="B58">
+      <c r="C58">
         <v>44</v>
       </c>
-      <c r="C58">
+      <c r="D58">
         <v>2.8899999999999999E-2</v>
       </c>
-      <c r="D58">
+      <c r="E58">
         <v>5.8500000000000003E-2</v>
       </c>
-      <c r="E58">
+      <c r="F58">
         <v>2E-3</v>
-      </c>
-      <c r="F58">
-        <v>450</v>
       </c>
       <c r="G58">
         <v>450</v>
@@ -6155,39 +6291,42 @@
         <v>450</v>
       </c>
       <c r="I58">
-        <v>0</v>
+        <v>450</v>
       </c>
       <c r="J58">
         <v>0</v>
       </c>
       <c r="K58">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L58">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M58">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N58">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="59" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59">
         <v>15</v>
       </c>
-      <c r="B59">
+      <c r="C59">
         <v>45</v>
       </c>
-      <c r="C59">
-        <v>0</v>
-      </c>
       <c r="D59">
+        <v>0</v>
+      </c>
+      <c r="E59">
         <v>0.1042</v>
       </c>
-      <c r="E59">
-        <v>0</v>
-      </c>
       <c r="F59">
-        <v>282</v>
+        <v>0</v>
       </c>
       <c r="G59">
         <v>282</v>
@@ -6196,39 +6335,42 @@
         <v>282</v>
       </c>
       <c r="I59">
+        <v>282</v>
+      </c>
+      <c r="J59">
         <v>0.95499999999999996</v>
       </c>
-      <c r="J59">
-        <v>0</v>
-      </c>
       <c r="K59">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L59">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M59">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N59">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="60" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60">
         <v>14</v>
       </c>
-      <c r="B60">
+      <c r="C60">
         <v>46</v>
       </c>
-      <c r="C60">
-        <v>0</v>
-      </c>
       <c r="D60">
+        <v>0</v>
+      </c>
+      <c r="E60">
         <v>7.3499999999999996E-2</v>
       </c>
-      <c r="E60">
-        <v>0</v>
-      </c>
       <c r="F60">
-        <v>400</v>
+        <v>0</v>
       </c>
       <c r="G60">
         <v>400</v>
@@ -6237,39 +6379,42 @@
         <v>400</v>
       </c>
       <c r="I60">
+        <v>400</v>
+      </c>
+      <c r="J60">
         <v>0.9</v>
       </c>
-      <c r="J60">
-        <v>0</v>
-      </c>
       <c r="K60">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L60">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M60">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N60">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="61" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61">
         <v>46</v>
       </c>
-      <c r="B61">
+      <c r="C61">
         <v>47</v>
       </c>
-      <c r="C61">
+      <c r="D61">
         <v>2.3E-2</v>
       </c>
-      <c r="D61">
+      <c r="E61">
         <v>6.8000000000000005E-2</v>
       </c>
-      <c r="E61">
+      <c r="F61">
         <v>3.2000000000000002E-3</v>
-      </c>
-      <c r="F61">
-        <v>409</v>
       </c>
       <c r="G61">
         <v>409</v>
@@ -6278,39 +6423,42 @@
         <v>409</v>
       </c>
       <c r="I61">
-        <v>0</v>
+        <v>409</v>
       </c>
       <c r="J61">
         <v>0</v>
       </c>
       <c r="K61">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L61">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M61">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N61">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="62" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A62">
+        <v>61</v>
+      </c>
+      <c r="B62">
         <v>47</v>
       </c>
-      <c r="B62">
+      <c r="C62">
         <v>48</v>
       </c>
-      <c r="C62">
+      <c r="D62">
         <v>1.8200000000000001E-2</v>
       </c>
-      <c r="D62">
+      <c r="E62">
         <v>2.3300000000000001E-2</v>
       </c>
-      <c r="E62">
-        <v>0</v>
-      </c>
       <c r="F62">
-        <v>993</v>
+        <v>0</v>
       </c>
       <c r="G62">
         <v>993</v>
@@ -6319,39 +6467,42 @@
         <v>993</v>
       </c>
       <c r="I62">
-        <v>0</v>
+        <v>993</v>
       </c>
       <c r="J62">
         <v>0</v>
       </c>
       <c r="K62">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L62">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M62">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N62">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="63" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A63">
+        <v>62</v>
+      </c>
+      <c r="B63">
         <v>48</v>
       </c>
-      <c r="B63">
+      <c r="C63">
         <v>49</v>
       </c>
-      <c r="C63">
+      <c r="D63">
         <v>8.3400000000000002E-2</v>
       </c>
-      <c r="D63">
+      <c r="E63">
         <v>0.129</v>
       </c>
-      <c r="E63">
+      <c r="F63">
         <v>4.7999999999999996E-3</v>
-      </c>
-      <c r="F63">
-        <v>191</v>
       </c>
       <c r="G63">
         <v>191</v>
@@ -6360,39 +6511,42 @@
         <v>191</v>
       </c>
       <c r="I63">
-        <v>0</v>
+        <v>191</v>
       </c>
       <c r="J63">
         <v>0</v>
       </c>
       <c r="K63">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L63">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M63">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N63">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="64" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64">
         <v>49</v>
       </c>
-      <c r="B64">
+      <c r="C64">
         <v>50</v>
       </c>
-      <c r="C64">
+      <c r="D64">
         <v>8.0100000000000005E-2</v>
       </c>
-      <c r="D64">
+      <c r="E64">
         <v>0.128</v>
       </c>
-      <c r="E64">
-        <v>0</v>
-      </c>
       <c r="F64">
-        <v>195</v>
+        <v>0</v>
       </c>
       <c r="G64">
         <v>195</v>
@@ -6401,39 +6555,42 @@
         <v>195</v>
       </c>
       <c r="I64">
-        <v>0</v>
+        <v>195</v>
       </c>
       <c r="J64">
         <v>0</v>
       </c>
       <c r="K64">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L64">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M64">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N64">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="65" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A65">
+        <v>64</v>
+      </c>
+      <c r="B65">
         <v>50</v>
       </c>
-      <c r="B65">
+      <c r="C65">
         <v>51</v>
       </c>
-      <c r="C65">
+      <c r="D65">
         <v>0.1386</v>
       </c>
-      <c r="D65">
+      <c r="E65">
         <v>0.22</v>
       </c>
-      <c r="E65">
-        <v>0</v>
-      </c>
       <c r="F65">
-        <v>113</v>
+        <v>0</v>
       </c>
       <c r="G65">
         <v>113</v>
@@ -6442,39 +6599,42 @@
         <v>113</v>
       </c>
       <c r="I65">
-        <v>0</v>
+        <v>113</v>
       </c>
       <c r="J65">
         <v>0</v>
       </c>
       <c r="K65">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L65">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M65">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N65">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="66" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A66">
+        <v>65</v>
+      </c>
+      <c r="B66">
         <v>10</v>
       </c>
-      <c r="B66">
+      <c r="C66">
         <v>51</v>
       </c>
-      <c r="C66">
-        <v>0</v>
-      </c>
       <c r="D66">
+        <v>0</v>
+      </c>
+      <c r="E66">
         <v>7.1199999999999999E-2</v>
       </c>
-      <c r="E66">
-        <v>0</v>
-      </c>
       <c r="F66">
-        <v>412</v>
+        <v>0</v>
       </c>
       <c r="G66">
         <v>412</v>
@@ -6483,39 +6643,42 @@
         <v>412</v>
       </c>
       <c r="I66">
+        <v>412</v>
+      </c>
+      <c r="J66">
         <v>0.93</v>
       </c>
-      <c r="J66">
-        <v>0</v>
-      </c>
       <c r="K66">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L66">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M66">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="67" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N66">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="67" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A67">
+        <v>66</v>
+      </c>
+      <c r="B67">
         <v>13</v>
       </c>
-      <c r="B67">
+      <c r="C67">
         <v>49</v>
       </c>
-      <c r="C67">
-        <v>0</v>
-      </c>
       <c r="D67">
+        <v>0</v>
+      </c>
+      <c r="E67">
         <v>0.191</v>
       </c>
-      <c r="E67">
-        <v>0</v>
-      </c>
       <c r="F67">
-        <v>154</v>
+        <v>0</v>
       </c>
       <c r="G67">
         <v>154</v>
@@ -6524,39 +6687,42 @@
         <v>154</v>
       </c>
       <c r="I67">
+        <v>154</v>
+      </c>
+      <c r="J67">
         <v>0.89500000000000002</v>
       </c>
-      <c r="J67">
-        <v>0</v>
-      </c>
       <c r="K67">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L67">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M67">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="68" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N67">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="68" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A68">
+        <v>67</v>
+      </c>
+      <c r="B68">
         <v>29</v>
       </c>
-      <c r="B68">
+      <c r="C68">
         <v>52</v>
       </c>
-      <c r="C68">
+      <c r="D68">
         <v>0.14419999999999999</v>
       </c>
-      <c r="D68">
+      <c r="E68">
         <v>0.187</v>
       </c>
-      <c r="E68">
-        <v>0</v>
-      </c>
       <c r="F68">
-        <v>125</v>
+        <v>0</v>
       </c>
       <c r="G68">
         <v>125</v>
@@ -6565,39 +6731,42 @@
         <v>125</v>
       </c>
       <c r="I68">
-        <v>0</v>
+        <v>125</v>
       </c>
       <c r="J68">
         <v>0</v>
       </c>
       <c r="K68">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L68">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M68">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="69" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N68">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="69" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A69">
+        <v>68</v>
+      </c>
+      <c r="B69">
         <v>52</v>
       </c>
-      <c r="B69">
+      <c r="C69">
         <v>53</v>
       </c>
-      <c r="C69">
+      <c r="D69">
         <v>7.6200000000000004E-2</v>
       </c>
-      <c r="D69">
+      <c r="E69">
         <v>9.8400000000000001E-2</v>
       </c>
-      <c r="E69">
-        <v>0</v>
-      </c>
       <c r="F69">
-        <v>236</v>
+        <v>0</v>
       </c>
       <c r="G69">
         <v>236</v>
@@ -6606,39 +6775,42 @@
         <v>236</v>
       </c>
       <c r="I69">
-        <v>0</v>
+        <v>236</v>
       </c>
       <c r="J69">
         <v>0</v>
       </c>
       <c r="K69">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L69">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M69">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="70" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N69">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="70" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A70">
+        <v>69</v>
+      </c>
+      <c r="B70">
         <v>53</v>
       </c>
-      <c r="B70">
+      <c r="C70">
         <v>54</v>
       </c>
-      <c r="C70">
+      <c r="D70">
         <v>0.18779999999999999</v>
       </c>
-      <c r="D70">
+      <c r="E70">
         <v>0.23200000000000001</v>
       </c>
-      <c r="E70">
-        <v>0</v>
-      </c>
       <c r="F70">
-        <v>99</v>
+        <v>0</v>
       </c>
       <c r="G70">
         <v>99</v>
@@ -6647,39 +6819,42 @@
         <v>99</v>
       </c>
       <c r="I70">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="J70">
         <v>0</v>
       </c>
       <c r="K70">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L70">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M70">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="71" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N70">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="71" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A71">
+        <v>70</v>
+      </c>
+      <c r="B71">
         <v>54</v>
       </c>
-      <c r="B71">
+      <c r="C71">
         <v>55</v>
       </c>
-      <c r="C71">
+      <c r="D71">
         <v>0.17319999999999999</v>
       </c>
-      <c r="D71">
+      <c r="E71">
         <v>0.22650000000000001</v>
       </c>
-      <c r="E71">
-        <v>0</v>
-      </c>
       <c r="F71">
-        <v>103</v>
+        <v>0</v>
       </c>
       <c r="G71">
         <v>103</v>
@@ -6688,39 +6863,42 @@
         <v>103</v>
       </c>
       <c r="I71">
-        <v>0</v>
+        <v>103</v>
       </c>
       <c r="J71">
         <v>0</v>
       </c>
       <c r="K71">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L71">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M71">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N71">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="72" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A72">
+        <v>71</v>
+      </c>
+      <c r="B72">
         <v>11</v>
       </c>
-      <c r="B72">
+      <c r="C72">
         <v>43</v>
       </c>
-      <c r="C72">
-        <v>0</v>
-      </c>
       <c r="D72">
+        <v>0</v>
+      </c>
+      <c r="E72">
         <v>0.153</v>
       </c>
-      <c r="E72">
-        <v>0</v>
-      </c>
       <c r="F72">
-        <v>192</v>
+        <v>0</v>
       </c>
       <c r="G72">
         <v>192</v>
@@ -6729,39 +6907,42 @@
         <v>192</v>
       </c>
       <c r="I72">
+        <v>192</v>
+      </c>
+      <c r="J72">
         <v>0.95799999999999996</v>
       </c>
-      <c r="J72">
-        <v>0</v>
-      </c>
       <c r="K72">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L72">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M72">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="73" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N72">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="73" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A73">
+        <v>72</v>
+      </c>
+      <c r="B73">
         <v>44</v>
       </c>
-      <c r="B73">
+      <c r="C73">
         <v>45</v>
       </c>
-      <c r="C73">
+      <c r="D73">
         <v>6.2399999999999997E-2</v>
       </c>
-      <c r="D73">
+      <c r="E73">
         <v>0.1242</v>
       </c>
-      <c r="E73">
+      <c r="F73">
         <v>4.0000000000000001E-3</v>
-      </c>
-      <c r="F73">
-        <v>212</v>
       </c>
       <c r="G73">
         <v>212</v>
@@ -6770,39 +6951,42 @@
         <v>212</v>
       </c>
       <c r="I73">
-        <v>0</v>
+        <v>212</v>
       </c>
       <c r="J73">
         <v>0</v>
       </c>
       <c r="K73">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L73">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M73">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="74" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N73">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="74" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A74">
+        <v>73</v>
+      </c>
+      <c r="B74">
         <v>40</v>
       </c>
-      <c r="B74">
+      <c r="C74">
         <v>56</v>
       </c>
-      <c r="C74">
-        <v>0</v>
-      </c>
       <c r="D74">
+        <v>0</v>
+      </c>
+      <c r="E74">
         <v>1.1950000000000001</v>
       </c>
-      <c r="E74">
-        <v>0</v>
-      </c>
       <c r="F74">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="G74">
         <v>25</v>
@@ -6811,39 +6995,42 @@
         <v>25</v>
       </c>
       <c r="I74">
+        <v>25</v>
+      </c>
+      <c r="J74">
         <v>0.95799999999999996</v>
       </c>
-      <c r="J74">
-        <v>0</v>
-      </c>
       <c r="K74">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L74">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M74">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="75" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N74">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="75" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A75">
+        <v>74</v>
+      </c>
+      <c r="B75">
         <v>56</v>
       </c>
-      <c r="B75">
+      <c r="C75">
         <v>41</v>
       </c>
-      <c r="C75">
+      <c r="D75">
         <v>0.55300000000000005</v>
       </c>
-      <c r="D75">
+      <c r="E75">
         <v>0.54900000000000004</v>
       </c>
-      <c r="E75">
-        <v>0</v>
-      </c>
       <c r="F75">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="G75">
         <v>38</v>
@@ -6852,39 +7039,42 @@
         <v>38</v>
       </c>
       <c r="I75">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="J75">
         <v>0</v>
       </c>
       <c r="K75">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L75">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M75">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="76" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N75">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="76" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A76">
+        <v>75</v>
+      </c>
+      <c r="B76">
         <v>56</v>
       </c>
-      <c r="B76">
+      <c r="C76">
         <v>42</v>
       </c>
-      <c r="C76">
+      <c r="D76">
         <v>0.21249999999999999</v>
       </c>
-      <c r="D76">
+      <c r="E76">
         <v>0.35399999999999998</v>
       </c>
-      <c r="E76">
-        <v>0</v>
-      </c>
       <c r="F76">
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="G76">
         <v>72</v>
@@ -6893,39 +7083,42 @@
         <v>72</v>
       </c>
       <c r="I76">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="J76">
         <v>0</v>
       </c>
       <c r="K76">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L76">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M76">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="77" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N76">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="77" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A77">
+        <v>76</v>
+      </c>
+      <c r="B77">
         <v>39</v>
       </c>
-      <c r="B77">
+      <c r="C77">
         <v>57</v>
       </c>
-      <c r="C77">
-        <v>0</v>
-      </c>
       <c r="D77">
+        <v>0</v>
+      </c>
+      <c r="E77">
         <v>1.355</v>
       </c>
-      <c r="E77">
-        <v>0</v>
-      </c>
       <c r="F77">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="G77">
         <v>22</v>
@@ -6934,39 +7127,42 @@
         <v>22</v>
       </c>
       <c r="I77">
+        <v>22</v>
+      </c>
+      <c r="J77">
         <v>0.98</v>
       </c>
-      <c r="J77">
-        <v>0</v>
-      </c>
       <c r="K77">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L77">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M77">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="78" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N77">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="78" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A78">
+        <v>77</v>
+      </c>
+      <c r="B78">
         <v>57</v>
       </c>
-      <c r="B78">
+      <c r="C78">
         <v>56</v>
       </c>
-      <c r="C78">
+      <c r="D78">
         <v>0.17399999999999999</v>
       </c>
-      <c r="D78">
+      <c r="E78">
         <v>0.26</v>
       </c>
-      <c r="E78">
-        <v>0</v>
-      </c>
       <c r="F78">
-        <v>94</v>
+        <v>0</v>
       </c>
       <c r="G78">
         <v>94</v>
@@ -6975,39 +7171,42 @@
         <v>94</v>
       </c>
       <c r="I78">
-        <v>0</v>
+        <v>94</v>
       </c>
       <c r="J78">
         <v>0</v>
       </c>
       <c r="K78">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L78">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M78">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="79" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N78">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="79" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A79">
+        <v>78</v>
+      </c>
+      <c r="B79">
         <v>38</v>
       </c>
-      <c r="B79">
+      <c r="C79">
         <v>49</v>
       </c>
-      <c r="C79">
+      <c r="D79">
         <v>0.115</v>
       </c>
-      <c r="D79">
+      <c r="E79">
         <v>0.17699999999999999</v>
       </c>
-      <c r="E79">
+      <c r="F79">
         <v>3.0000000000000001E-3</v>
-      </c>
-      <c r="F79">
-        <v>139</v>
       </c>
       <c r="G79">
         <v>139</v>
@@ -7016,39 +7215,42 @@
         <v>139</v>
       </c>
       <c r="I79">
-        <v>0</v>
+        <v>139</v>
       </c>
       <c r="J79">
         <v>0</v>
       </c>
       <c r="K79">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L79">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M79">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="80" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N79">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="80" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A80">
+        <v>79</v>
+      </c>
+      <c r="B80">
         <v>38</v>
       </c>
-      <c r="B80">
+      <c r="C80">
         <v>48</v>
       </c>
-      <c r="C80">
+      <c r="D80">
         <v>3.1199999999999999E-2</v>
       </c>
-      <c r="D80">
+      <c r="E80">
         <v>4.82E-2</v>
       </c>
-      <c r="E80">
-        <v>0</v>
-      </c>
       <c r="F80">
-        <v>511</v>
+        <v>0</v>
       </c>
       <c r="G80">
         <v>511</v>
@@ -7057,39 +7259,42 @@
         <v>511</v>
       </c>
       <c r="I80">
-        <v>0</v>
+        <v>511</v>
       </c>
       <c r="J80">
         <v>0</v>
       </c>
       <c r="K80">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L80">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M80">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="81" spans="1:13" x14ac:dyDescent="0.3">
+        <v>-30</v>
+      </c>
+      <c r="N80">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="81" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A81">
+        <v>80</v>
+      </c>
+      <c r="B81">
         <v>9</v>
       </c>
-      <c r="B81">
+      <c r="C81">
         <v>55</v>
       </c>
-      <c r="C81">
-        <v>0</v>
-      </c>
       <c r="D81">
+        <v>0</v>
+      </c>
+      <c r="E81">
         <v>0.1205</v>
       </c>
-      <c r="E81">
-        <v>0</v>
-      </c>
       <c r="F81">
-        <v>244</v>
+        <v>0</v>
       </c>
       <c r="G81">
         <v>244</v>
@@ -7098,18 +7303,21 @@
         <v>244</v>
       </c>
       <c r="I81">
+        <v>244</v>
+      </c>
+      <c r="J81">
         <v>0.94</v>
       </c>
-      <c r="J81">
-        <v>0</v>
-      </c>
       <c r="K81">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L81">
-        <v>-30</v>
+        <v>1</v>
       </c>
       <c r="M81">
+        <v>-30</v>
+      </c>
+      <c r="N81">
         <v>30</v>
       </c>
     </row>

</xml_diff>